<commit_message>
Updated 4B and Added 4C excerices
</commit_message>
<xml_diff>
--- a/week-01/Ex4A_GTrends.xlsx
+++ b/week-01/Ex4A_GTrends.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Brandon\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{B9B62C9F-F6F1-439B-8B9D-250BD5712802}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BBC055F9-F8E4-4C8C-95CA-0C99B6CF455C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{49F1C08D-31FF-4AB3-807B-E395AC2E4217}"/>
   </bookViews>
@@ -18,7 +18,20 @@
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">GTrends_milkshake_hamburger_202!$A$1:$E$1</definedName>
   </definedNames>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -1068,6 +1081,7 @@
   <dimension ref="A1:H52"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
+    <col min="1" max="1" width="11.140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.7109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="29.5703125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="28.7109375" bestFit="1" customWidth="1"/>

</xml_diff>